<commit_message>
task133 realism repair 3: remaining term pinned under payment pauses and past maturity, Office theme parts, development-sample chronology, working-document wording and AASB 9 clauses, extract residue (overseas addresses, unrecorded reasons, weekly status batch), measured docx statistics, service-account register; allowance unchanged at AUD 13,773,000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task133/golden/ecl_allowance_2026Q3.xlsx
+++ b/task133/golden/ecl_allowance_2026Q3.xlsx
@@ -98,7 +98,7 @@
     <t>Stage 2: 30 or more days past due, a hardship arrangement in force on 30 September 2026 (start on or before, end on or after, not cancelled), or a behaviour score 60 or more points below origination on scorecard v4; v3 origination scores converted as 1.12 x v3 - 18, rounded (section 2 and the June 2024 migration note).</t>
   </si>
   <si>
-    <t>PD(k) is (C(a+k) - C(a+k-1)) / (1 - C(a)) on the PLPD-2026.06 curve for the loan's product, where a is the number of monthly repayments fallen due by 30 September: the curve runs from origination, and a performing loan has already come through its first a months. A loan past its contractual maturity outside stage 3 has one remaining month (section 3.2), the last month of its product's curve.</t>
+    <t>PD(k) is (C(a+k) - C(a+k-1)) / (1 - C(a)) on the PLPD-2026.06 curve for the loan's product, where a is the number of monthly repayments fallen due by 30 September, repayment dates in a payment pause included: the curve runs from origination, and a performing loan has already come through its first a months. A loan past its contractual maturity outside stage 3 is in the final month of its term with one month remaining (section 3.2), the last month of its product's curve.</t>
   </si>
   <si>
     <t>EAD re-amortises the current balance over the remaining term at the contract rate; months discounted at the contract rate; LGD 70 per cent PL36, 76 per cent PL60 (sections 3.3 to 3.5).</t>
@@ -230,34 +230,34 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -265,9 +265,9 @@
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -294,14 +294,32 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -328,6 +346,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -339,166 +375,142 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 

</xml_diff>

<commit_message>
task133 loop 1: rebuilt pack, goldens and target.zip
Fifteen input files (five new: the June quarter-end extract, the scoring
runs, the 2023-24 defaults, the receipts ledger, the debt-sale schedule);
distractors are now the roll-rate workbook and the write-off file. Golden
allowance AUD 13,160,000 (stage 1 10,563,000, stage 2 2,597,000); the
workbook carries the realised-loss grid and the migration counts, the
deck's second slide the stacked migration chart. Two scratch rebuilds are
byte-identical to target/, golden/ and target.zip.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task133/golden/ecl_allowance_2026Q3.xlsx
+++ b/task133/golden/ecl_allowance_2026Q3.xlsx
@@ -9,21 +9,21 @@
   </bookViews>
   <sheets>
     <sheet name="Allowance" sheetId="1" r:id="rId1"/>
-    <sheet name="Stage and product" sheetId="2" r:id="rId2"/>
-    <sheet name="By drawdown year" sheetId="3" r:id="rId3"/>
-    <sheet name="Notes" sheetId="4" r:id="rId4"/>
+    <sheet name="Realised LGD" sheetId="2" r:id="rId2"/>
+    <sheet name="Stage migration" sheetId="3" r:id="rId3"/>
+    <sheet name="Method" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
   <si>
     <t>Personal loans (PL36, PL60): collective ECL allowance at 30 September 2026</t>
   </si>
   <si>
-    <t>Credit Risk Reporting, 9 October 2026. CRM-ECL-04 v4.1; scenarios approved 18 September 2026.</t>
+    <t>Credit Risk Reporting, 9 October 2026. CRM-ECL-04 v4.2; scenarios approved 18 September 2026.</t>
   </si>
   <si>
     <t>Collective ECL allowance (AUD)</t>
@@ -35,79 +35,100 @@
     <t>Stage 2 allowance (AUD)</t>
   </si>
   <si>
+    <t>Loans in stage 1</t>
+  </si>
+  <si>
+    <t>Loans in stage 2</t>
+  </si>
+  <si>
+    <t>Loans in stage 3, assessed under CRM-ECL-06</t>
+  </si>
+  <si>
     <t>Probability-weighted PD multiplier</t>
   </si>
   <si>
-    <t>Loans in stage 3, outside the collective model</t>
-  </si>
-  <si>
-    <t>Stage</t>
+    <t>Source: loan system extract ECL_QE_BOOK at close of business 30 September 2026 (run 1 October); PLPD-2026.06 curve and development sample; Q1 FY27 scenario sheet.</t>
+  </si>
+  <si>
+    <t>2023-24 defaults: share of the balance at default not recovered, at 30 September 2026 (CRM-ECL-04 3.3)</t>
   </si>
   <si>
     <t>Product</t>
   </si>
   <si>
+    <t>Quarter of default</t>
+  </si>
+  <si>
     <t>Loans</t>
   </si>
   <si>
-    <t>Gross carrying amount (AUD)</t>
-  </si>
-  <si>
-    <t>Allowance (AUD)</t>
-  </si>
-  <si>
-    <t>Coverage (%)</t>
+    <t>Balance at default (AUD)</t>
+  </si>
+  <si>
+    <t>Realised loss (%)</t>
+  </si>
+  <si>
+    <t>LGD in use (%)</t>
+  </si>
+  <si>
+    <t>PL36</t>
+  </si>
+  <si>
+    <t>Jul to Sep 2023</t>
+  </si>
+  <si>
+    <t>Oct to Dec 2023</t>
+  </si>
+  <si>
+    <t>Jan to Mar 2024</t>
+  </si>
+  <si>
+    <t>Apr to Jun 2024</t>
+  </si>
+  <si>
+    <t>PL60</t>
+  </si>
+  <si>
+    <t>Loans in stage 1 or 2 at 30 June 2026: where they stand at 30 September 2026</t>
+  </si>
+  <si>
+    <t>Stage at 30 June</t>
   </si>
   <si>
     <t>Stage 1</t>
   </si>
   <si>
-    <t>PL36</t>
-  </si>
-  <si>
-    <t>PL60</t>
-  </si>
-  <si>
     <t>Stage 2</t>
   </si>
   <si>
-    <t>Drawdown year</t>
-  </si>
-  <si>
-    <t>PL36 allowance (AUD)</t>
-  </si>
-  <si>
-    <t>PL60 allowance (AUD)</t>
-  </si>
-  <si>
-    <t>2023 and earlier</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
-    <t>2025</t>
-  </si>
-  <si>
-    <t>2026</t>
-  </si>
-  <si>
-    <t>Scope: PL36 and PL60 loans open in the loan system at close of business 30 September 2026; loans 90 or more days past due are stage 3 and sit under CRM-ECL-06 (CRM-ECL-04 section 1).</t>
-  </si>
-  <si>
-    <t>Stage 2: 30 or more days past due, a hardship arrangement in force on 30 September 2026 (start on or before, end on or after, not cancelled), or a behaviour score 60 or more points below origination on scorecard v4; v3 origination scores converted as 1.12 x v3 - 18, rounded (section 2 and the June 2024 migration note).</t>
-  </si>
-  <si>
-    <t>PD(k) is (C(a+k) - C(a+k-1)) / (1 - C(a)) on the PLPD-2026.06 curve for the loan's product, where a is the number of monthly repayments fallen due by 30 September, repayment dates in a payment pause included: the curve runs from origination, and a performing loan has already come through its first a months. A loan past its contractual maturity outside stage 3 is in the final month of its term with one month remaining (section 3.2), the last month of its product's curve.</t>
-  </si>
-  <si>
-    <t>EAD re-amortises the current balance over the remaining term at the contract rate; months discounted at the contract rate; LGD 70 per cent PL36, 76 per cent PL60 (sections 3.3 to 3.5).</t>
-  </si>
-  <si>
-    <t>Scenario weights 55 / 30 / 15 per cent on PD multipliers 1.00 / 1.30 / 0.80 give a weighted multiplier of 1.0600 (section 4).</t>
-  </si>
-  <si>
-    <t>Amounts are rounded to the nearest thousand dollars from unrounded loan-level results, so rows may not add exactly.</t>
+    <t>Stage 3</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>Loans at 30 June</t>
+  </si>
+  <si>
+    <t>Stage at 30 September under CRM-ECL-04 section 2; closed means repaid, settled or written off by then.</t>
+  </si>
+  <si>
+    <t>Scope: PL36 and PL60 loans open at close of business 30 September 2026. Loans 90 or more days past due are stage 3 and are assessed under CRM-ECL-06.</t>
+  </si>
+  <si>
+    <t>Stage 2: 30 or more days past due, a hardship arrangement in force on the date (start to end, both included, not from the day it is cancelled), or a behaviour score 60 or more points below origination on v4 from the month-end run on the position at the date; v3 origination scores converted as 1.12 x v3 - 18, rounded. At 30 June the June month-end run (made 1 July) supplies the scores.</t>
+  </si>
+  <si>
+    <t>PD(k): the PLPD-2026.06 curve gives, for every loan drawn in the development window, the share defaulted by each month on book. A loan a months on book that is still open and has not defaulted takes (C(a+k) - C(a+k-1)) / S(a), where S(a) is the share of the development sample still open and never defaulted at the end of month a (1 - C(a) less the share repaid in full by then). Stage 2 PD carries the 2.4 scalar. A loan past its maturity outside stage 3 has one month remaining (3.2).</t>
+  </si>
+  <si>
+    <t>EAD re-amortises the current balance over the remaining term at the contract rate; each month is discounted at the contract rate; LGD 70 per cent PL36, 76 per cent PL60; scenarios 55 / 30 / 15 per cent on multipliers 1.00 / 1.30 / 0.80 (weighted 1.06).</t>
+  </si>
+  <si>
+    <t>Realised loss (3.3): receipts after default to 30 September 2026 from the Collections receipts file, plus each sold account's share of the March 2026 sale (face value at cut-off x 3.85 cents), each taken at the end of the month received and discounted to the default month end at the contract rate; cured loans lose nothing.</t>
+  </si>
+  <si>
+    <t>Amounts are rounded to the nearest thousand dollars from loan-level results, so stage amounts may not add exactly.</t>
   </si>
 </sst>
 </file>
@@ -116,9 +137,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +166,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -185,20 +214,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -516,11 +547,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FECEF707-7CC3-4602-830C-06AB2E21172D}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="46.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -538,7 +569,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4">
-        <v>13773000</v>
+        <v>13160000</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -546,7 +577,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5">
-        <v>10933000</v>
+        <v>10563000</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -554,23 +585,44 @@
         <v>4</v>
       </c>
       <c r="B6" s="5">
-        <v>2840000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="6">
-        <v>1.06</v>
+        <v>2597000</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6">
+        <v>37288</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B9" s="6">
+        <v>3266</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6">
         <v>343</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -581,115 +633,200 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A7C7CA4-85C6-4ECD-8D37-C64D13DD0CB9}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="26.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="8" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="7">
-        <v>17109</v>
-      </c>
-      <c r="D2" s="5">
-        <v>138349000</v>
-      </c>
-      <c r="E2" s="5">
-        <v>3202000</v>
-      </c>
-      <c r="F2" s="9">
-        <v>2.31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="E3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="7">
-        <v>20180</v>
-      </c>
-      <c r="D3" s="5">
-        <v>330436000</v>
-      </c>
-      <c r="E3" s="5">
-        <v>7731000</v>
-      </c>
-      <c r="F3" s="9">
-        <v>2.34</v>
+      <c r="F3" s="9" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="7">
-        <v>1421</v>
-      </c>
-      <c r="D4" s="5">
-        <v>11728000</v>
-      </c>
-      <c r="E4" s="5">
-        <v>681000</v>
-      </c>
-      <c r="F4" s="9">
-        <v>5.81</v>
+        <v>18</v>
+      </c>
+      <c r="C4" s="6">
+        <v>142</v>
+      </c>
+      <c r="D4" s="10">
+        <v>1445693.9</v>
+      </c>
+      <c r="E4" s="11">
+        <v>67.9</v>
+      </c>
+      <c r="F4" s="12">
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="7">
-        <v>1844</v>
-      </c>
-      <c r="D5" s="5">
-        <v>28735000</v>
-      </c>
-      <c r="E5" s="5">
-        <v>2159000</v>
-      </c>
-      <c r="F5" s="9">
-        <v>7.51</v>
+        <v>19</v>
+      </c>
+      <c r="C5" s="6">
+        <v>139</v>
+      </c>
+      <c r="D5" s="10">
+        <v>1489194.03</v>
+      </c>
+      <c r="E5" s="11">
+        <v>65.8</v>
+      </c>
+      <c r="F5" s="12">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="6">
+        <v>164</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1825983.96</v>
+      </c>
+      <c r="E6" s="11">
+        <v>70.7</v>
+      </c>
+      <c r="F6" s="12">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="6">
+        <v>144</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1486050.53</v>
+      </c>
+      <c r="E7" s="11">
+        <v>70.9</v>
+      </c>
+      <c r="F7" s="12">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="6">
+        <v>119</v>
+      </c>
+      <c r="D8" s="10">
+        <v>3016811.56</v>
+      </c>
+      <c r="E8" s="11">
+        <v>70.4</v>
+      </c>
+      <c r="F8" s="12">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="6">
+        <v>126</v>
+      </c>
+      <c r="D9" s="10">
+        <v>2751515.5</v>
+      </c>
+      <c r="E9" s="11">
+        <v>77.3</v>
+      </c>
+      <c r="F9" s="12">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="6">
+        <v>158</v>
+      </c>
+      <c r="D10" s="10">
+        <v>3274739.94</v>
+      </c>
+      <c r="E10" s="11">
+        <v>73.5</v>
+      </c>
+      <c r="F10" s="12">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="6">
+        <v>156</v>
+      </c>
+      <c r="D11" s="10">
+        <v>3434027.51</v>
+      </c>
+      <c r="E11" s="11">
+        <v>79.3</v>
+      </c>
+      <c r="F11" s="12">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -700,72 +837,146 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ADD81C2-E051-4BAF-8CFB-BB5EEB6DBEDA}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="5">
-        <v>5000</v>
-      </c>
-      <c r="C2" s="5">
-        <v>641000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="5">
-        <v>159000</v>
-      </c>
-      <c r="C3" s="5">
-        <v>1073000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="6">
+        <v>14470</v>
+      </c>
+      <c r="D4" s="6">
+        <v>680</v>
+      </c>
+      <c r="E4" s="6">
+        <v>42</v>
+      </c>
+      <c r="F4" s="6">
+        <v>1586</v>
+      </c>
+      <c r="G4" s="6">
+        <v>16778</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="6">
+        <v>468</v>
+      </c>
+      <c r="D5" s="6">
+        <v>658</v>
+      </c>
+      <c r="E5" s="6">
+        <v>115</v>
+      </c>
+      <c r="F5" s="6">
+        <v>123</v>
+      </c>
+      <c r="G5" s="6">
+        <v>1364</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="5">
-        <v>940000</v>
-      </c>
-      <c r="C4" s="5">
-        <v>2412000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="5">
-        <v>2779000</v>
-      </c>
-      <c r="C5" s="5">
-        <v>5763000</v>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="6">
+        <v>17724</v>
+      </c>
+      <c r="D6" s="6">
+        <v>831</v>
+      </c>
+      <c r="E6" s="6">
+        <v>46</v>
+      </c>
+      <c r="F6" s="6">
+        <v>1180</v>
+      </c>
+      <c r="G6" s="6">
+        <v>19781</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="6">
+        <v>560</v>
+      </c>
+      <c r="D7" s="6">
+        <v>942</v>
+      </c>
+      <c r="E7" s="6">
+        <v>140</v>
+      </c>
+      <c r="F7" s="6">
+        <v>112</v>
+      </c>
+      <c r="G7" s="6">
+        <v>1754</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -774,37 +985,37 @@
   <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="125.7109375" customWidth="1"/>
+    <col min="1" max="1" width="120.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>24</v>
+      <c r="A1" s="13" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>25</v>
+      <c r="A2" s="13" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>26</v>
+      <c r="A3" s="13" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>27</v>
+      <c r="A4" s="13" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>28</v>
+      <c r="A5" s="13" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>29</v>
+      <c r="A6" s="13" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>